<commit_message>
Populate institutional model with Visa historical financials and KPIs
</commit_message>
<xml_diff>
--- a/model/Visa_Institutional_Model_v2.xlsx
+++ b/model/Visa_Institutional_Model_v2.xlsx
@@ -40,7 +40,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -130,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -157,6 +160,21 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -547,13 +565,6 @@
           <t>Visa Institutional Equity Research Model V2</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -561,13 +572,6 @@
           <t>FIG / Payments Coverage Model</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -813,13 +817,6 @@
           <t>Operating Expense Build</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -828,13 +825,6 @@
           <t>Forecast expenses and operating leverage.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -1000,11 +990,21 @@
           <t>G&amp;A / Other</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="B10" s="10" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>10497</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>11653</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>12331</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>16006</v>
+      </c>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
@@ -1015,23 +1015,23 @@
           <t>Total Operating Expenses</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="13">
         <f>SUM(B6:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="13">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="13">
         <f>SUM(D6:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="13">
         <f>SUM(E6:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="13">
         <f>SUM(F6:F10)</f>
         <v/>
       </c>
@@ -1054,23 +1054,23 @@
           <t>Operating Income</t>
         </is>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="13">
         <f>B5-B11</f>
         <v/>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="13">
         <f>C5-C11</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="13">
         <f>D5-D11</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="13">
         <f>E5-E11</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="13">
         <f>F5-F11</f>
         <v/>
       </c>
@@ -1093,23 +1093,23 @@
           <t>Operating Margin</t>
         </is>
       </c>
-      <c r="B13" s="8">
+      <c r="B13" s="14">
         <f>B12/B5</f>
         <v/>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="14">
         <f>C12/C5</f>
         <v/>
       </c>
-      <c r="D13" s="8">
+      <c r="D13" s="14">
         <f>D12/D5</f>
         <v/>
       </c>
-      <c r="E13" s="8">
+      <c r="E13" s="14">
         <f>E12/E5</f>
         <v/>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="14">
         <f>F12/F5</f>
         <v/>
       </c>
@@ -1164,13 +1164,6 @@
           <t>Operating Margin Walk</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1178,13 +1171,6 @@
           <t>Bridge current margin to forecast margin.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -1385,13 +1371,6 @@
           <t>Tax, D&amp;A, Capex, and Working Capital</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -1400,13 +1379,6 @@
           <t>Core free cash flow forecast assumptions.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -1760,13 +1732,6 @@
           <t>Unlevered Free Cash Flow</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -1775,13 +1740,6 @@
           <t>DCF cash flow build.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -2150,13 +2108,6 @@
           <t>Share Count and Buybacks</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -2165,13 +2116,6 @@
           <t>Model EPS accretion from capital return.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -2486,13 +2430,6 @@
           <t>DCF Valuation</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -2501,13 +2438,6 @@
           <t>Intrinsic valuation using unlevered free cash flow.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -2949,13 +2879,6 @@
           <t>Trading Comparable Company Analysis</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
@@ -2966,13 +2889,6 @@
           <t>Benchmark Visa against payments peers.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
@@ -3335,13 +3251,6 @@
           <t>Precedent Transaction Analysis</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
@@ -3352,13 +3261,6 @@
           <t>Payments M&amp;A valuation context.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
@@ -3661,13 +3563,6 @@
           <t>Sum-of-the-Parts Valuation</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -3675,13 +3570,6 @@
           <t>Separate core network, VAS, and money movement value pools.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -3887,13 +3775,6 @@
           <t>Scenario Manager</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -3901,13 +3782,6 @@
           <t>Driver-based severe downside, bear, base, and bull cases.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -4102,7 +3976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4125,13 +3999,6 @@
           <t>Sources</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4139,13 +4006,6 @@
           <t>All major figures should be traceable to filings, transcripts, or public market data.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -4360,6 +4220,70 @@
       </c>
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Company Filing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Visa annual reports / Form 10-K</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FY2021-FY2025</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Historical financials</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>data/processed/visa_historical_financials_source_backed.csv</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Populated into model by script</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Company Filing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Visa annual reports / Form 10-K</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FY2021-FY2025</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Operating KPIs</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>data/processed/visa_operating_kpis_source_backed.csv</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Populated into model by script</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4399,13 +4323,6 @@
           <t>Sensitivity Tables</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4413,13 +4330,6 @@
           <t>DCF and valuation sensitivity outputs.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -4663,13 +4573,6 @@
           <t>Consensus Bridge</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4677,13 +4580,6 @@
           <t>Compare project estimates with consensus expectations.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -4895,13 +4791,6 @@
           <t>Output Dashboard</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4909,13 +4798,6 @@
           <t>Recruiter-friendly model summary.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -5105,13 +4987,6 @@
           <t>Charts</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5119,13 +4994,6 @@
           <t>Placeholder sheet for report-ready chart outputs.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -5301,13 +5169,6 @@
           <t>Model Checks</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5315,13 +5176,6 @@
           <t>Quality-control checks for model integrity.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -5456,13 +5310,6 @@
           <t>Print Package</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5470,13 +5317,6 @@
           <t>Sections to print/export for appendix.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -5638,13 +5478,6 @@
           <t>Setup and Control</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5652,13 +5485,6 @@
           <t>Central assumptions for valuation and scenarios.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
@@ -5888,13 +5714,6 @@
           <t>Historical Financials</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -5903,13 +5722,6 @@
           <t>Input reported historical financials and forecast core line items.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -5976,11 +5788,21 @@
           <t>Net Revenue</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="B5" s="10" t="n">
+        <v>24105</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>29310</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>32653</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>35926</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>40000</v>
+      </c>
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="8" t="n"/>
@@ -5991,20 +5813,20 @@
           <t>YoY Revenue Growth</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7">
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="11">
         <f>D5/C5-1</f>
         <v/>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="11">
         <f>E5/D5-1</f>
         <v/>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="11">
         <f>F5/E5-1</f>
         <v/>
       </c>
@@ -6027,11 +5849,21 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="B7" s="10" t="n">
+        <v>8301</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>10497</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>11653</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>12331</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>16006</v>
+      </c>
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="8" t="n"/>
@@ -6042,25 +5874,20 @@
           <t>Operating Income</t>
         </is>
       </c>
-      <c r="B8" s="7">
-        <f>B5-B7</f>
-        <v/>
-      </c>
-      <c r="C8" s="7">
-        <f>C5-C7</f>
-        <v/>
-      </c>
-      <c r="D8" s="7">
-        <f>D5-D7</f>
-        <v/>
-      </c>
-      <c r="E8" s="7">
-        <f>E5-E7</f>
-        <v/>
-      </c>
-      <c r="F8" s="7">
-        <f>F5-F7</f>
-        <v/>
+      <c r="B8" s="10" t="n">
+        <v>15804</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>18813</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>21000</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>23595</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>23994</v>
       </c>
       <c r="G8" s="8">
         <f>G5-G7</f>
@@ -6081,25 +5908,20 @@
           <t>Operating Margin</t>
         </is>
       </c>
-      <c r="B9" s="7">
-        <f>B8/B5</f>
-        <v/>
-      </c>
-      <c r="C9" s="7">
-        <f>C8/C5</f>
-        <v/>
-      </c>
-      <c r="D9" s="7">
-        <f>D8/D5</f>
-        <v/>
-      </c>
-      <c r="E9" s="7">
-        <f>E8/E5</f>
-        <v/>
-      </c>
-      <c r="F9" s="7">
-        <f>F8/F5</f>
-        <v/>
+      <c r="B9" s="11" t="n">
+        <v>0.6556000000000001</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0.6418</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>0.6431</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>0.6567000000000001</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0.5999</v>
       </c>
       <c r="G9" s="8">
         <f>G8/G5</f>
@@ -6120,11 +5942,21 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="B10" s="10" t="n">
+        <v>12311</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>14957</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>17273</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>19743</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>20058</v>
+      </c>
       <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
@@ -6135,11 +5967,21 @@
           <t>Diluted EPS</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="B11" s="12" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>10.2</v>
+      </c>
       <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
@@ -6150,11 +5992,21 @@
           <t>Operating Cash Flow</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="B12" s="10" t="n">
+        <v>15227</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>18849</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>20755</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>19950</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>23059</v>
+      </c>
       <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
@@ -6165,11 +6017,21 @@
           <t>Capital Expenditures</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="B13" s="10" t="n">
+        <v>705</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>970</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>1059</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>1257</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>1482</v>
+      </c>
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
@@ -6180,25 +6042,20 @@
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="B14" s="7">
-        <f>B12-B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="7">
-        <f>C12-C13</f>
-        <v/>
-      </c>
-      <c r="D14" s="7">
-        <f>D12-D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="7">
-        <f>E12-E13</f>
-        <v/>
-      </c>
-      <c r="F14" s="7">
-        <f>F12-F13</f>
-        <v/>
+      <c r="B14" s="10" t="n">
+        <v>14522</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>17879</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>19696</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>18693</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>21577</v>
       </c>
       <c r="G14" s="8">
         <f>G12-G13</f>
@@ -6219,11 +6076,21 @@
           <t>Diluted Shares</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
+      <c r="B15" s="12" t="n">
+        <v>2186.678507992895</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>2136.714285714286</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>2086.111111111111</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>2029.085303186022</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>1966.470588235294</v>
+      </c>
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
@@ -6266,13 +6133,6 @@
           <t>Payments KPI History</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
     </row>
@@ -6282,13 +6142,6 @@
           <t>Operating KPIs specific to networks and payments.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
     </row>
@@ -6362,11 +6215,21 @@
           <t>Payments Volume</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="B5" s="12" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>14.2</v>
+      </c>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
@@ -6382,11 +6245,21 @@
           <t>Processed Transactions</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="B6" s="12" t="n">
+        <v>164.7</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="D6" s="12" t="n">
+        <v>212.6</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <v>233.8</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>257.5</v>
+      </c>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
@@ -6422,11 +6295,21 @@
           <t>Credentials</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="B8" s="12" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>4.9</v>
+      </c>
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
@@ -6462,11 +6345,21 @@
           <t>Gross Revenue Yield</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="B10" s="11" t="n">
+        <v>0.003122307692307692</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0.003414224137931035</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>0.003654471544715447</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0.003764393939393939</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0.00392612676056338</v>
+      </c>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
@@ -6482,11 +6375,21 @@
           <t>Net Revenue Yield</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
+      <c r="B11" s="11" t="n">
+        <v>0.002317788461538461</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>0.002526724137931034</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>0.002654715447154472</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>0.002721666666666667</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0.002816901408450704</v>
+      </c>
       <c r="G11" s="7" t="n"/>
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
@@ -6502,11 +6405,21 @@
           <t>Client Incentives / Gross Revenue</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
+      <c r="B12" s="11" t="n">
+        <v>0.2576681448632668</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>0.2599419265244287</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>0.2735706340378198</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.2769973837794325</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.2825240802855554</v>
+      </c>
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
@@ -6522,11 +6435,17 @@
           <t>VAS Revenue</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>8800</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>10900</v>
+      </c>
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
@@ -6542,11 +6461,17 @@
           <t>VAS % of Net Revenue</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n">
+        <v>0.2205004134382752</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.2449479485609308</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.2725</v>
+      </c>
       <c r="G14" s="7" t="n"/>
       <c r="H14" s="7" t="n"/>
       <c r="I14" s="7" t="n"/>
@@ -6594,13 +6519,6 @@
           <t>Revenue Build</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -6609,13 +6527,6 @@
           <t>Driver-based revenue forecast.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -6682,11 +6593,21 @@
           <t>Service Revenue</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="B5" s="10" t="n">
+        <v>11475</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>13361</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>14826</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>16114</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>17539</v>
+      </c>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
@@ -6697,11 +6618,21 @@
           <t>Data Processing Revenue</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="7" t="n"/>
+      <c r="B6" s="10" t="n">
+        <v>12792</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>14438</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>16007</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>17714</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>19993</v>
+      </c>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
@@ -6712,11 +6643,21 @@
           <t>International Transaction Revenue</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="B7" s="10" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>9815</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>11638</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>12665</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>14166</v>
+      </c>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
@@ -6727,11 +6668,21 @@
           <t>Other Revenue</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
+      <c r="B8" s="10" t="n">
+        <v>1675</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>1991</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>2479</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>3197</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>4053</v>
+      </c>
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
       <c r="I8" s="7" t="n"/>
@@ -6742,23 +6693,23 @@
           <t>Gross Revenue</t>
         </is>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="13">
         <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="13">
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="13">
         <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="13">
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="13">
         <f>SUM(F5:F8)</f>
         <v/>
       </c>
@@ -6781,11 +6732,21 @@
           <t>Client Incentives</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
+      <c r="B10" s="10" t="n">
+        <v>8367</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>10295</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>12297</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>13764</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>15751</v>
+      </c>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
@@ -6796,23 +6757,23 @@
           <t>Net Revenue</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="13">
         <f>B9-B10</f>
         <v/>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="13">
         <f>C9-C10</f>
         <v/>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="13">
         <f>D9-D10</f>
         <v/>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="13">
         <f>E9-E10</f>
         <v/>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="13">
         <f>F9-F10</f>
         <v/>
       </c>
@@ -6835,20 +6796,20 @@
           <t>Net Revenue Growth</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8">
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14">
         <f>C11/B11-1</f>
         <v/>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="14">
         <f>D11/C11-1</f>
         <v/>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="14">
         <f>E11/D11-1</f>
         <v/>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="14">
         <f>F11/E11-1</f>
         <v/>
       </c>
@@ -6903,13 +6864,6 @@
           <t>Client Incentives</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -6918,13 +6872,6 @@
           <t>Analyze partner economics and take-rate pressure.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -7192,7 +7139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7215,13 +7162,6 @@
           <t>Value-Added Services Model</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -7230,13 +7170,6 @@
           <t>Analyze Visa's services growth runway.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -7303,11 +7236,17 @@
           <t>VAS Revenue</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n"/>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>8800</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>10900</v>
+      </c>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
@@ -7318,20 +7257,20 @@
           <t>VAS Growth</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8">
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="14">
         <f>D5/C5-1</f>
         <v/>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="14">
         <f>E5/D5-1</f>
         <v/>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="14">
         <f>F5/E5-1</f>
         <v/>
       </c>
@@ -7354,23 +7293,23 @@
           <t>Net Revenue</t>
         </is>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="13">
         <f>'06_Revenue_Build'!B11</f>
         <v/>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="13">
         <f>'06_Revenue_Build'!C11</f>
         <v/>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="13">
         <f>'06_Revenue_Build'!D11</f>
         <v/>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="13">
         <f>'06_Revenue_Build'!E11</f>
         <v/>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="13">
         <f>'06_Revenue_Build'!F11</f>
         <v/>
       </c>
@@ -7393,23 +7332,23 @@
           <t>VAS % of Net Revenue</t>
         </is>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="14">
         <f>B5/B7</f>
         <v/>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="14">
         <f>C5/C7</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="14">
         <f>D5/D7</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="14">
         <f>E5/E7</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="14">
         <f>F5/F7</f>
         <v/>
       </c>
@@ -7480,6 +7419,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -7518,13 +7458,6 @@
           <t>Cross-Border Model</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
@@ -7533,13 +7466,6 @@
           <t>High-yield international revenue sensitivity.</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -7657,11 +7583,21 @@
           <t>International Transaction Revenue</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
+      <c r="B7" s="10" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>9815</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>11638</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>12665</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>14166</v>
+      </c>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
@@ -7672,20 +7608,20 @@
           <t>International Revenue Growth</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8">
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="14">
         <f>C7/B7-1</f>
         <v/>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="14">
         <f>D7/C7-1</f>
         <v/>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="14">
         <f>E7/D7-1</f>
         <v/>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="14">
         <f>F7/E7-1</f>
         <v/>
       </c>

</xml_diff>